<commit_message>
슬라임(11001) max_deck_count 20으로 수정
</commit_message>
<xml_diff>
--- a/GameDesign/Storage/SampleData/Card.xlsx
+++ b/GameDesign/Storage/SampleData/Card.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="26827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wnsal\Ttakji_lab-mobile_development_dep\GameDesign\Storage\SampleData\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Git\Ttakji_lab-mobile_development_dep\GameDesign\Storage\SampleData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F220A08E-D28A-4A65-B8E6-4150823A1752}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{58EB29B5-6AF8-4268-B67D-9CB4C4B138F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28590" yWindow="-1905" windowWidth="16410" windowHeight="18315" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Card" sheetId="1" r:id="rId1"/>
@@ -560,7 +560,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -614,8 +614,15 @@
       <charset val="129"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="맑은 고딕"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="12">
+  <fills count="13">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -678,6 +685,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="8"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -746,7 +759,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
@@ -774,6 +787,7 @@
     <xf numFmtId="0" fontId="0" fillId="10" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="9" borderId="0" xfId="2" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="6" fillId="11" borderId="0" xfId="3" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="7" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="20% - 강조색1" xfId="2" builtinId="30"/>
@@ -1226,8 +1240,8 @@
       <c r="C4" t="s">
         <v>4</v>
       </c>
-      <c r="D4">
-        <v>2</v>
+      <c r="D4" s="19">
+        <v>20</v>
       </c>
       <c r="E4" t="s">
         <v>114</v>

</xml_diff>

<commit_message>
CardUnit, CardSkill 에 desc 필드 추가
기존에는 주석처리 되어있었음
</commit_message>
<xml_diff>
--- a/GameDesign/Storage/SampleData/Card.xlsx
+++ b/GameDesign/Storage/SampleData/Card.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\git\Ttakji_lab-mobile_development_dep\GameDesign\Storage\SampleData\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Git\Ttakji_lab-mobile_development_dep\GameDesign\Storage\SampleData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ABF1CD01-97C5-48C4-9527-55D91D7F9BCE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E14C2658-AAF2-4C72-8251-DF020AC1487A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-105" yWindow="0" windowWidth="29010" windowHeight="15585" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Card" sheetId="1" r:id="rId1"/>
@@ -492,10 +492,6 @@
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
-    <t>string(128)</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
     <t>pow300이하 적 유닛 1장 파괴(승점X)</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
@@ -559,6 +555,10 @@
   </si>
   <si>
     <t>Assets/Resources/card_img/Mana_Potion.png</t>
+  </si>
+  <si>
+    <t>desc</t>
+    <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
 </file>
@@ -745,7 +745,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
@@ -767,12 +767,10 @@
     <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="8" borderId="0" xfId="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="6" fillId="10" borderId="0" xfId="3" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="2" applyFill="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="2" applyFill="1" applyBorder="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="4">
@@ -827,7 +825,7 @@
   <tableColumns count="20">
     <tableColumn id="1" xr3:uid="{E1C732DB-5275-4BF3-8215-44D4B7F98F34}" name="id"/>
     <tableColumn id="2" xr3:uid="{AA754E55-C3C2-4F3C-A9D2-8AE9F68682DC}" name="#name"/>
-    <tableColumn id="4" xr3:uid="{4265547F-DD0C-47BC-9461-16331FFAC9E4}" name="#desc"/>
+    <tableColumn id="4" xr3:uid="{4265547F-DD0C-47BC-9461-16331FFAC9E4}" name="desc"/>
     <tableColumn id="3" xr3:uid="{7032B4B8-4205-47FC-9689-BC42E6DF9D37}" name="prize"/>
     <tableColumn id="28" xr3:uid="{29A4D6B9-AB36-40F4-B8A4-C9B6870FC42E}" name="arts_cost"/>
     <tableColumn id="27" xr3:uid="{A9A2C876-6B0F-4AFE-A5DA-1F3B17D95FB6}" name="power"/>
@@ -872,7 +870,7 @@
   <tableColumns count="9">
     <tableColumn id="1" xr3:uid="{8D4780BB-DB0E-4DB7-98EE-B9656815F7E3}" name="id"/>
     <tableColumn id="2" xr3:uid="{930486ED-C78F-4EB0-A0FF-6750226B4381}" name="#name"/>
-    <tableColumn id="9" xr3:uid="{F058E14E-AA4C-45AF-9E9C-7C8B9FA6C2D8}" name="#desc"/>
+    <tableColumn id="9" xr3:uid="{F058E14E-AA4C-45AF-9E9C-7C8B9FA6C2D8}" name="desc"/>
     <tableColumn id="3" xr3:uid="{E1E06BC9-C21F-44D1-AEEB-BA85426B8332}" name="skill_cost"/>
     <tableColumn id="4" xr3:uid="{B1591891-D015-470D-84EF-F5BCE8D0B39A}" name="use_condition_type"/>
     <tableColumn id="5" xr3:uid="{679497A7-A7A1-4666-85D3-098B0B4B862D}" name="use_condition_value1"/>
@@ -1167,7 +1165,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F15"/>
+  <dimension ref="A1:E14"/>
   <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="11" bestFit="1" customWidth="1"/>
@@ -1177,12 +1175,12 @@
     <col min="6" max="7" width="18.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="33" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" ht="33" x14ac:dyDescent="0.3">
       <c r="C1" s="4" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -1199,7 +1197,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
         <v>6</v>
       </c>
@@ -1216,211 +1214,192 @@
         <v>17</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A4" s="13">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A4">
         <v>11001</v>
       </c>
-      <c r="B4" s="13" t="s">
+      <c r="B4" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="13" t="s">
+      <c r="C4" t="s">
         <v>4</v>
       </c>
-      <c r="D4" s="13">
+      <c r="D4">
         <v>20</v>
       </c>
-      <c r="E4" s="13" t="s">
+      <c r="E4" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A5">
+        <v>11002</v>
+      </c>
+      <c r="B5" t="s">
+        <v>100</v>
+      </c>
+      <c r="C5" t="s">
+        <v>4</v>
+      </c>
+      <c r="D5">
+        <v>2</v>
+      </c>
+      <c r="E5" t="s">
         <v>123</v>
       </c>
-      <c r="F4" s="13"/>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A5" s="13">
-        <v>11002</v>
-      </c>
-      <c r="B5" s="13" t="s">
-        <v>100</v>
-      </c>
-      <c r="C5" s="13" t="s">
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A6">
+        <v>11003</v>
+      </c>
+      <c r="B6" t="s">
+        <v>101</v>
+      </c>
+      <c r="C6" t="s">
         <v>4</v>
       </c>
-      <c r="D5" s="13">
+      <c r="D6">
         <v>2</v>
       </c>
-      <c r="E5" s="13" t="s">
+      <c r="E6" t="s">
         <v>124</v>
       </c>
-      <c r="F5" s="13"/>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A6" s="13">
-        <v>11003</v>
-      </c>
-      <c r="B6" s="13" t="s">
-        <v>101</v>
-      </c>
-      <c r="C6" s="13" t="s">
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A7">
+        <v>11004</v>
+      </c>
+      <c r="B7" t="s">
+        <v>102</v>
+      </c>
+      <c r="C7" t="s">
         <v>4</v>
       </c>
-      <c r="D6" s="13">
+      <c r="D7">
         <v>2</v>
       </c>
-      <c r="E6" s="13" t="s">
+      <c r="E7" t="s">
         <v>125</v>
       </c>
-      <c r="F6" s="13"/>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A7" s="13">
-        <v>11004</v>
-      </c>
-      <c r="B7" s="13" t="s">
-        <v>102</v>
-      </c>
-      <c r="C7" s="13" t="s">
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A8">
+        <v>11005</v>
+      </c>
+      <c r="B8" t="s">
+        <v>103</v>
+      </c>
+      <c r="C8" t="s">
         <v>4</v>
       </c>
-      <c r="D7" s="13">
+      <c r="D8">
         <v>2</v>
       </c>
-      <c r="E7" s="13" t="s">
+      <c r="E8" t="s">
         <v>126</v>
       </c>
-      <c r="F7" s="13"/>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A8" s="13">
-        <v>11005</v>
-      </c>
-      <c r="B8" s="13" t="s">
-        <v>103</v>
-      </c>
-      <c r="C8" s="13" t="s">
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A9">
+        <v>11006</v>
+      </c>
+      <c r="B9" t="s">
+        <v>104</v>
+      </c>
+      <c r="C9" t="s">
         <v>4</v>
       </c>
-      <c r="D8" s="13">
+      <c r="D9">
         <v>2</v>
       </c>
-      <c r="E8" s="13" t="s">
+      <c r="E9" t="s">
         <v>127</v>
       </c>
-      <c r="F8" s="13"/>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A9" s="13">
-        <v>11006</v>
-      </c>
-      <c r="B9" s="13" t="s">
-        <v>104</v>
-      </c>
-      <c r="C9" s="13" t="s">
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A10">
+        <v>11007</v>
+      </c>
+      <c r="B10" t="s">
+        <v>119</v>
+      </c>
+      <c r="C10" t="s">
         <v>4</v>
       </c>
-      <c r="D9" s="13">
+      <c r="D10">
         <v>2</v>
       </c>
-      <c r="E9" s="13" t="s">
+      <c r="E10" t="s">
         <v>128</v>
       </c>
-      <c r="F9" s="13"/>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A10" s="13">
-        <v>11007</v>
-      </c>
-      <c r="B10" s="13" t="s">
-        <v>120</v>
-      </c>
-      <c r="C10" s="13" t="s">
-        <v>4</v>
-      </c>
-      <c r="D10" s="13">
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A11">
+        <v>21001</v>
+      </c>
+      <c r="B11" t="s">
+        <v>13</v>
+      </c>
+      <c r="C11" t="s">
+        <v>14</v>
+      </c>
+      <c r="D11">
         <v>2</v>
       </c>
-      <c r="E10" s="13" t="s">
+      <c r="E11" t="s">
         <v>129</v>
       </c>
-      <c r="F10" s="13"/>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A11" s="13">
-        <v>21001</v>
-      </c>
-      <c r="B11" s="13" t="s">
-        <v>13</v>
-      </c>
-      <c r="C11" s="13" t="s">
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A12" s="13">
+        <v>21002</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="C12" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="D11" s="13">
+      <c r="D12" s="14">
         <v>2</v>
       </c>
-      <c r="E11" s="13" t="s">
+      <c r="E12" t="s">
         <v>130</v>
       </c>
-      <c r="F11" s="13"/>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A12" s="14">
-        <v>21002</v>
-      </c>
-      <c r="B12" s="15" t="s">
-        <v>85</v>
-      </c>
-      <c r="C12" s="15" t="s">
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A13">
+        <v>21003</v>
+      </c>
+      <c r="B13" t="s">
+        <v>86</v>
+      </c>
+      <c r="C13" t="s">
         <v>14</v>
       </c>
-      <c r="D12" s="16">
+      <c r="D13">
         <v>2</v>
       </c>
-      <c r="E12" s="13" t="s">
+      <c r="E13" t="s">
         <v>131</v>
       </c>
-      <c r="F12" s="13"/>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A13" s="13">
-        <v>21003</v>
-      </c>
-      <c r="B13" s="13" t="s">
-        <v>86</v>
-      </c>
-      <c r="C13" s="13" t="s">
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A14" s="15">
+        <v>21004</v>
+      </c>
+      <c r="B14" s="16" t="s">
+        <v>87</v>
+      </c>
+      <c r="C14" s="16" t="s">
         <v>14</v>
       </c>
-      <c r="D13" s="13">
+      <c r="D14" s="17">
         <v>2</v>
       </c>
-      <c r="E13" s="13" t="s">
+      <c r="E14" t="s">
         <v>132</v>
       </c>
-      <c r="F13" s="13"/>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A14" s="17">
-        <v>21004</v>
-      </c>
-      <c r="B14" s="18" t="s">
-        <v>87</v>
-      </c>
-      <c r="C14" s="18" t="s">
-        <v>14</v>
-      </c>
-      <c r="D14" s="19">
-        <v>2</v>
-      </c>
-      <c r="E14" s="13" t="s">
-        <v>133</v>
-      </c>
-      <c r="F14" s="13"/>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A15" s="13"/>
-      <c r="B15" s="13"/>
-      <c r="C15" s="13"/>
-      <c r="D15" s="13"/>
-      <c r="E15" s="13"/>
-      <c r="F15" s="13"/>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
@@ -1498,10 +1477,10 @@
         <v>84</v>
       </c>
       <c r="C2" t="s">
-        <v>15</v>
+        <v>133</v>
       </c>
       <c r="D2" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="E2" t="s">
         <v>18</v>
@@ -1995,10 +1974,10 @@
         <v>11007</v>
       </c>
       <c r="B10" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="C10" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="D10">
         <v>1</v>
@@ -2192,7 +2171,7 @@
         <v>84</v>
       </c>
       <c r="C2" t="s">
-        <v>15</v>
+        <v>133</v>
       </c>
       <c r="D2" s="1" t="s">
         <v>56</v>
@@ -2221,7 +2200,7 @@
         <v>7</v>
       </c>
       <c r="C3" s="12" t="s">
-        <v>114</v>
+        <v>17</v>
       </c>
       <c r="D3" s="10" t="s">
         <v>11</v>
@@ -2250,7 +2229,7 @@
         <v>13</v>
       </c>
       <c r="C4" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D4" s="2">
         <v>1</v>
@@ -2279,7 +2258,7 @@
         <v>85</v>
       </c>
       <c r="C5" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="D5">
         <v>1</v>
@@ -2308,7 +2287,7 @@
         <v>86</v>
       </c>
       <c r="C6" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="D6">
         <v>1</v>
@@ -2337,7 +2316,7 @@
         <v>87</v>
       </c>
       <c r="C7" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="D7">
         <v>1</v>
@@ -2697,10 +2676,10 @@
         <v>210018</v>
       </c>
       <c r="B11" t="s">
+        <v>119</v>
+      </c>
+      <c r="C11" t="s">
         <v>120</v>
-      </c>
-      <c r="C11" t="s">
-        <v>121</v>
       </c>
       <c r="D11" t="s">
         <v>98</v>

</xml_diff>

<commit_message>
Damege->Damage 오타 수정 및 DeckHighOrEqual->DeckMoreOrEqual 변경
</commit_message>
<xml_diff>
--- a/GameDesign/Storage/SampleData/Card.xlsx
+++ b/GameDesign/Storage/SampleData/Card.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="26827"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Git\Ttakji_lab-mobile_development_dep\GameDesign\Storage\SampleData\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wnsal\Ttakji_lab-mobile_development_dep\GameDesign\Storage\SampleData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E14C2658-AAF2-4C72-8251-DF020AC1487A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{051CE217-CBC0-4C46-9E1C-56324EA9A78D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="0" windowWidth="29010" windowHeight="15585" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Card" sheetId="1" r:id="rId1"/>
@@ -433,9 +433,6 @@
     <t>OwnMana</t>
   </si>
   <si>
-    <t>DeckHighOrEqual</t>
-  </si>
-  <si>
     <t>레드슬라임</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
@@ -484,10 +481,6 @@
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
-    <t>DamegeToUnit</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
     <t>적 1장 데미지 200(승점X)</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
@@ -520,10 +513,6 @@
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
-    <t>등장시 자신은 이번턴 마나 1을 획득한다.</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
     <t>Assets/Resources/card_img/u_slime.png</t>
   </si>
   <si>
@@ -558,6 +547,18 @@
   </si>
   <si>
     <t>desc</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>DamageToUnit</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>DeckMoreOrEqual</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>등장 시 자신은 이번턴 마나 1을 획득한다.</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
@@ -1228,7 +1229,7 @@
         <v>20</v>
       </c>
       <c r="E4" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.3">
@@ -1236,7 +1237,7 @@
         <v>11002</v>
       </c>
       <c r="B5" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C5" t="s">
         <v>4</v>
@@ -1245,7 +1246,7 @@
         <v>2</v>
       </c>
       <c r="E5" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.3">
@@ -1253,7 +1254,7 @@
         <v>11003</v>
       </c>
       <c r="B6" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="C6" t="s">
         <v>4</v>
@@ -1262,7 +1263,7 @@
         <v>2</v>
       </c>
       <c r="E6" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.3">
@@ -1270,7 +1271,7 @@
         <v>11004</v>
       </c>
       <c r="B7" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C7" t="s">
         <v>4</v>
@@ -1279,7 +1280,7 @@
         <v>2</v>
       </c>
       <c r="E7" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.3">
@@ -1287,7 +1288,7 @@
         <v>11005</v>
       </c>
       <c r="B8" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C8" t="s">
         <v>4</v>
@@ -1296,7 +1297,7 @@
         <v>2</v>
       </c>
       <c r="E8" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.3">
@@ -1304,7 +1305,7 @@
         <v>11006</v>
       </c>
       <c r="B9" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C9" t="s">
         <v>4</v>
@@ -1313,7 +1314,7 @@
         <v>2</v>
       </c>
       <c r="E9" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.3">
@@ -1321,7 +1322,7 @@
         <v>11007</v>
       </c>
       <c r="B10" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="C10" t="s">
         <v>4</v>
@@ -1330,7 +1331,7 @@
         <v>2</v>
       </c>
       <c r="E10" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.3">
@@ -1347,7 +1348,7 @@
         <v>2</v>
       </c>
       <c r="E11" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.3">
@@ -1364,7 +1365,7 @@
         <v>2</v>
       </c>
       <c r="E12" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.3">
@@ -1381,7 +1382,7 @@
         <v>2</v>
       </c>
       <c r="E13" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.3">
@@ -1398,7 +1399,7 @@
         <v>2</v>
       </c>
       <c r="E14" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
     </row>
   </sheetData>
@@ -1477,10 +1478,10 @@
         <v>84</v>
       </c>
       <c r="C2" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="D2" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="E2" t="s">
         <v>18</v>
@@ -1605,7 +1606,7 @@
         <v>3</v>
       </c>
       <c r="C4" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="D4">
         <v>1</v>
@@ -1664,10 +1665,10 @@
         <v>11002</v>
       </c>
       <c r="B5" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C5" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D5">
         <v>2</v>
@@ -1726,10 +1727,10 @@
         <v>11003</v>
       </c>
       <c r="B6" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="C6" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="D6">
         <v>3</v>
@@ -1788,10 +1789,10 @@
         <v>11004</v>
       </c>
       <c r="B7" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C7" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="D7">
         <v>1</v>
@@ -1850,10 +1851,10 @@
         <v>11005</v>
       </c>
       <c r="B8" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C8" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="D8">
         <v>1</v>
@@ -1912,10 +1913,10 @@
         <v>11006</v>
       </c>
       <c r="B9" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C9" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="D9">
         <v>2</v>
@@ -1974,10 +1975,10 @@
         <v>11007</v>
       </c>
       <c r="B10" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="C10" t="s">
-        <v>121</v>
+        <v>133</v>
       </c>
       <c r="D10">
         <v>1</v>
@@ -2171,7 +2172,7 @@
         <v>84</v>
       </c>
       <c r="C2" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="D2" s="1" t="s">
         <v>56</v>
@@ -2229,7 +2230,7 @@
         <v>13</v>
       </c>
       <c r="C4" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="D4" s="2">
         <v>1</v>
@@ -2258,7 +2259,7 @@
         <v>85</v>
       </c>
       <c r="C5" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="D5">
         <v>1</v>
@@ -2287,7 +2288,7 @@
         <v>86</v>
       </c>
       <c r="C6" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="D6">
         <v>1</v>
@@ -2316,7 +2317,7 @@
         <v>87</v>
       </c>
       <c r="C7" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="D7">
         <v>1</v>
@@ -2478,7 +2479,7 @@
         <v>-1</v>
       </c>
       <c r="F5" t="s">
-        <v>99</v>
+        <v>132</v>
       </c>
       <c r="G5">
         <v>1</v>
@@ -2571,7 +2572,7 @@
         <v>210015</v>
       </c>
       <c r="B8" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C8" t="s">
         <v>93</v>
@@ -2583,7 +2584,7 @@
         <v>-1</v>
       </c>
       <c r="F8" t="s">
-        <v>99</v>
+        <v>132</v>
       </c>
       <c r="G8">
         <v>1</v>
@@ -2606,10 +2607,10 @@
         <v>210016</v>
       </c>
       <c r="B9" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C9" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="D9" t="s">
         <v>69</v>
@@ -2627,7 +2628,7 @@
         <v>-1</v>
       </c>
       <c r="I9" t="s">
-        <v>112</v>
+        <v>131</v>
       </c>
       <c r="J9">
         <v>0</v>
@@ -2641,10 +2642,10 @@
         <v>210017</v>
       </c>
       <c r="B10" t="s">
+        <v>103</v>
+      </c>
+      <c r="C10" t="s">
         <v>104</v>
-      </c>
-      <c r="C10" t="s">
-        <v>105</v>
       </c>
       <c r="D10" t="s">
         <v>69</v>
@@ -2676,10 +2677,10 @@
         <v>210018</v>
       </c>
       <c r="B11" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="C11" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="D11" t="s">
         <v>98</v>

</xml_diff>